<commit_message>
P0 quick closes: regenerate rate-bearing downloadable assets (xlsx/PDF/SVG) post-sweep, djh noise-filter entry, POST_LEDGER residue verified clean + header updated, proposal_engine committed (out/ gitignored), BADR gap figure 2026/27 patch
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property/web/public/resources/incorporation/incorporation-model.xlsx
+++ b/Property/web/public/resources/incorporation/incorporation-model.xlsx
@@ -364,10 +364,10 @@
     <t>Taxable dividend</t>
   </si>
   <si>
-    <t>Taxed at basic dividend rate (8.75%)</t>
-  </si>
-  <si>
-    <t>Taxed at higher dividend rate (33.75%)</t>
+    <t>Taxed at basic dividend rate (10.75%)</t>
+  </si>
+  <si>
+    <t>Taxed at higher dividend rate (35.75%)</t>
   </si>
   <si>
     <t>Taxed at additional dividend rate (39.35%)</t>
@@ -469,7 +469,7 @@
     <t xml:space="preserve">  £50,000, 25% from £250,000, marginal relief between). The company's money is not yours: unless you</t>
   </si>
   <si>
-    <t xml:space="preserve">  retain and reinvest it, drawing it out as dividends is taxed again (8.75% / 33.75% / 39.35%).</t>
+    <t xml:space="preserve">  retain and reinvest it, drawing it out as dividends is taxed again (10.75% / 35.75% / 39.35% for 2026/27).</t>
   </si>
   <si>
     <t>• Not modelled: company buy-to-let mortgage costs (usually higher), ATED on £500k+ dwellings (relieved</t>
@@ -1083,7 +1083,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="4">
-        <v>0.0875</v>
+        <v>0.1075</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -1091,7 +1091,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="4">
-        <v>0.3375</v>
+        <v>0.3575</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>